<commit_message>
updating LCSC BOM(Still remaing)
</commit_message>
<xml_diff>
--- a/Hardware-Designing/Deliverables/BOM/LCSC BOM.xlsx
+++ b/Hardware-Designing/Deliverables/BOM/LCSC BOM.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="14400" windowHeight="12345"/>
+    <workbookView windowWidth="24000" windowHeight="9795"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -436,14 +436,14 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="6">
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="&quot;$&quot;#,##0.00000"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    <numFmt numFmtId="179" formatCode="&quot;$&quot;#,##0.00000"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -504,6 +504,13 @@
     <font>
       <u/>
       <sz val="10"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
       <color theme="10"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -520,11 +527,93 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -543,57 +632,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color theme="10"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="15"/>
       <color theme="3"/>
@@ -602,50 +640,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -656,8 +662,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -684,73 +691,175 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -762,109 +871,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1046,17 +1053,28 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FF7F7F7F"/>
       </left>
       <right style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FF7F7F7F"/>
       </right>
       <top style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FF7F7F7F"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1076,35 +1094,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1126,11 +1120,24 @@
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="double">
-        <color theme="4"/>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1146,15 +1153,15 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -1164,133 +1171,133 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="20" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="28" fillId="24" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1361,22 +1368,19 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="5" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1389,16 +1393,16 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="179" fontId="10" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="11" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="177" fontId="10" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
@@ -1774,10 +1778,10 @@
       <c r="N1" s="3"/>
       <c r="O1" s="3"/>
       <c r="P1" s="3"/>
-      <c r="Q1" s="31"/>
-      <c r="R1" s="32"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="31"/>
       <c r="S1" s="2"/>
-      <c r="T1" s="32"/>
+      <c r="T1" s="31"/>
     </row>
     <row r="2" ht="16.5" spans="1:20">
       <c r="A2" s="4" t="s">
@@ -1834,14 +1838,14 @@
       <c r="R2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="S2" s="33" t="s">
+      <c r="S2" s="32" t="s">
         <v>19</v>
       </c>
       <c r="T2" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" ht="15.75" spans="1:20">
+    <row r="3" spans="1:20">
       <c r="A3" s="7">
         <v>1</v>
       </c>
@@ -1851,13 +1855,13 @@
       <c r="C3" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="40" t="s">
+      <c r="E3" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="40" t="s">
+      <c r="F3" s="39" t="s">
         <v>25</v>
       </c>
       <c r="G3" s="11" t="s">
@@ -1869,7 +1873,7 @@
       <c r="I3" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J3" s="41" t="s">
+      <c r="J3" s="40" t="s">
         <v>29</v>
       </c>
       <c r="K3" s="11">
@@ -1903,9 +1907,9 @@
         <f>R3*M3</f>
         <v>0.126</v>
       </c>
-      <c r="T3" s="34"/>
+      <c r="T3" s="33"/>
     </row>
-    <row r="4" ht="15.75" spans="1:20">
+    <row r="4" spans="1:20">
       <c r="A4" s="7">
         <v>2</v>
       </c>
@@ -1913,13 +1917,13 @@
       <c r="C4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="41" t="s">
+      <c r="E4" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="41" t="s">
+      <c r="F4" s="40" t="s">
         <v>33</v>
       </c>
       <c r="G4" s="11" t="s">
@@ -1931,7 +1935,7 @@
       <c r="I4" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J4" s="41" t="s">
+      <c r="J4" s="40" t="s">
         <v>35</v>
       </c>
       <c r="K4" s="11">
@@ -1965,7 +1969,7 @@
         <f t="shared" ref="S4:S21" si="3">R4*M4</f>
         <v>0.051</v>
       </c>
-      <c r="T4" s="34"/>
+      <c r="T4" s="33"/>
     </row>
     <row r="5" ht="16.5" spans="1:20">
       <c r="A5" s="7">
@@ -1974,16 +1978,16 @@
       <c r="B5" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="40" t="s">
+      <c r="D5" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="F5" s="40" t="s">
+      <c r="F5" s="39" t="s">
         <v>40</v>
       </c>
       <c r="G5" s="11" t="s">
@@ -2001,14 +2005,14 @@
       <c r="K5" s="11">
         <v>4</v>
       </c>
-      <c r="L5" s="26">
+      <c r="L5" s="22">
         <v>30</v>
       </c>
       <c r="M5" s="11">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N5" s="23" t="s">
+      <c r="N5" s="26" t="s">
         <v>30</v>
       </c>
       <c r="O5" s="24">
@@ -2029,7 +2033,7 @@
         <f t="shared" si="3"/>
         <v>1.264</v>
       </c>
-      <c r="T5" s="34"/>
+      <c r="T5" s="33"/>
     </row>
     <row r="6" ht="16.5" spans="1:20">
       <c r="A6" s="7">
@@ -2038,16 +2042,16 @@
       <c r="B6" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="43" t="s">
+      <c r="C6" s="42" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="41" t="s">
+      <c r="E6" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="F6" s="41" t="s">
+      <c r="F6" s="40" t="s">
         <v>48</v>
       </c>
       <c r="G6" s="11" t="s">
@@ -2093,9 +2097,9 @@
         <f t="shared" si="3"/>
         <v>0.562</v>
       </c>
-      <c r="T6" s="34"/>
+      <c r="T6" s="33"/>
     </row>
-    <row r="7" ht="15.75" spans="1:20">
+    <row r="7" spans="1:20">
       <c r="A7" s="7">
         <v>5</v>
       </c>
@@ -2105,13 +2109,13 @@
       <c r="C7" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="41" t="s">
+      <c r="E7" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="F7" s="41" t="s">
+      <c r="F7" s="40" t="s">
         <v>55</v>
       </c>
       <c r="G7" s="11" t="s">
@@ -2123,7 +2127,7 @@
       <c r="I7" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="J7" s="41" t="s">
+      <c r="J7" s="40" t="s">
         <v>59</v>
       </c>
       <c r="K7" s="14">
@@ -2136,7 +2140,7 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="N7" s="23" t="s">
+      <c r="N7" s="26" t="s">
         <v>30</v>
       </c>
       <c r="O7" s="24">
@@ -2157,23 +2161,23 @@
         <f t="shared" si="3"/>
         <v>0.03</v>
       </c>
-      <c r="T7" s="34"/>
+      <c r="T7" s="33"/>
     </row>
     <row r="8" ht="15.75" spans="1:20">
       <c r="A8" s="7">
         <v>6</v>
       </c>
       <c r="B8" s="15"/>
-      <c r="C8" s="43" t="s">
+      <c r="C8" s="42" t="s">
         <v>60</v>
       </c>
-      <c r="D8" s="41" t="s">
+      <c r="D8" s="40" t="s">
         <v>61</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="F8" s="41" t="s">
+      <c r="F8" s="40" t="s">
         <v>63</v>
       </c>
       <c r="G8" s="11" t="s">
@@ -2181,7 +2185,7 @@
       </c>
       <c r="H8" s="12"/>
       <c r="I8" s="11"/>
-      <c r="J8" s="41" t="s">
+      <c r="J8" s="40" t="s">
         <v>59</v>
       </c>
       <c r="K8" s="14">
@@ -2192,7 +2196,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N8" s="23"/>
+      <c r="N8" s="26"/>
       <c r="O8" s="24"/>
       <c r="P8" s="25">
         <f t="shared" si="1"/>
@@ -2207,23 +2211,23 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="T8" s="34"/>
+      <c r="T8" s="33"/>
     </row>
     <row r="9" ht="15.75" spans="1:20">
       <c r="A9" s="7">
         <v>7</v>
       </c>
       <c r="B9" s="15"/>
-      <c r="C9" s="43" t="s">
+      <c r="C9" s="42" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="41" t="s">
+      <c r="D9" s="40" t="s">
         <v>66</v>
       </c>
-      <c r="E9" s="41" t="s">
+      <c r="E9" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="F9" s="41" t="s">
+      <c r="F9" s="40" t="s">
         <v>67</v>
       </c>
       <c r="G9" s="11" t="s">
@@ -2235,7 +2239,7 @@
       <c r="I9" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J9" s="41" t="s">
+      <c r="J9" s="40" t="s">
         <v>70</v>
       </c>
       <c r="K9" s="14">
@@ -2248,7 +2252,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N9" s="23" t="s">
+      <c r="N9" s="26" t="s">
         <v>30</v>
       </c>
       <c r="O9" s="24">
@@ -2269,7 +2273,7 @@
         <f t="shared" si="3"/>
         <v>0.0075</v>
       </c>
-      <c r="T9" s="34"/>
+      <c r="T9" s="33"/>
     </row>
     <row r="10" ht="15.75" spans="1:20">
       <c r="A10" s="7">
@@ -2279,13 +2283,13 @@
       <c r="C10" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D10" s="41" t="s">
+      <c r="D10" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="E10" s="41" t="s">
+      <c r="E10" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="40" t="s">
         <v>73</v>
       </c>
       <c r="G10" s="11" t="s">
@@ -2297,7 +2301,7 @@
       <c r="I10" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="J10" s="41" t="s">
+      <c r="J10" s="40" t="s">
         <v>76</v>
       </c>
       <c r="K10" s="14">
@@ -2310,7 +2314,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N10" s="23" t="s">
+      <c r="N10" s="26" t="s">
         <v>30</v>
       </c>
       <c r="O10" s="24">
@@ -2331,7 +2335,7 @@
         <f t="shared" si="3"/>
         <v>0.0085</v>
       </c>
-      <c r="T10" s="34"/>
+      <c r="T10" s="33"/>
     </row>
     <row r="11" ht="15.75" spans="1:20">
       <c r="A11" s="7">
@@ -2341,13 +2345,13 @@
       <c r="C11" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="D11" s="40" t="s">
         <v>78</v>
       </c>
-      <c r="E11" s="41" t="s">
+      <c r="E11" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="41" t="s">
+      <c r="F11" s="40" t="s">
         <v>79</v>
       </c>
       <c r="G11" s="11" t="s">
@@ -2359,7 +2363,7 @@
       <c r="I11" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J11" s="41" t="s">
+      <c r="J11" s="40" t="s">
         <v>81</v>
       </c>
       <c r="K11" s="14">
@@ -2372,7 +2376,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="N11" s="23" t="s">
+      <c r="N11" s="26" t="s">
         <v>30</v>
       </c>
       <c r="O11" s="25">
@@ -2402,16 +2406,16 @@
       <c r="B12" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="C12" s="43" t="s">
+      <c r="C12" s="42" t="s">
         <v>83</v>
       </c>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="40" t="s">
         <v>84</v>
       </c>
       <c r="E12" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="F12" s="41" t="s">
+      <c r="F12" s="40" t="s">
         <v>85</v>
       </c>
       <c r="G12" s="11"/>
@@ -2428,7 +2432,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N12" s="28"/>
+      <c r="N12" s="26"/>
       <c r="O12" s="25"/>
       <c r="P12" s="25">
         <f t="shared" si="1"/>
@@ -2452,16 +2456,16 @@
       <c r="B13" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="C13" s="43" t="s">
+      <c r="C13" s="42" t="s">
         <v>87</v>
       </c>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="40" t="s">
         <v>88</v>
       </c>
       <c r="E13" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="F13" s="41" t="s">
+      <c r="F13" s="40" t="s">
         <v>89</v>
       </c>
       <c r="G13" s="11" t="s">
@@ -2486,7 +2490,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N13" s="23" t="s">
+      <c r="N13" s="26" t="s">
         <v>30</v>
       </c>
       <c r="O13" s="24">
@@ -2507,7 +2511,7 @@
         <f t="shared" si="3"/>
         <v>4.166</v>
       </c>
-      <c r="T13" s="35"/>
+      <c r="T13" s="34"/>
     </row>
     <row r="14" ht="15.75" spans="1:20">
       <c r="A14" s="7">
@@ -2516,16 +2520,16 @@
       <c r="B14" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="C14" s="43" t="s">
+      <c r="C14" s="42" t="s">
         <v>93</v>
       </c>
-      <c r="D14" s="41" t="s">
+      <c r="D14" s="40" t="s">
         <v>94</v>
       </c>
       <c r="E14" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="F14" s="41" t="s">
+      <c r="F14" s="40" t="s">
         <v>95</v>
       </c>
       <c r="G14" s="11" t="s">
@@ -2550,7 +2554,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N14" s="23" t="s">
+      <c r="N14" s="26" t="s">
         <v>30</v>
       </c>
       <c r="O14" s="25">
@@ -2571,23 +2575,23 @@
         <f t="shared" si="3"/>
         <v>25.5525</v>
       </c>
-      <c r="T14" s="36"/>
+      <c r="T14" s="35"/>
     </row>
     <row r="15" ht="15.75" spans="1:20">
       <c r="A15" s="7">
         <v>13</v>
       </c>
       <c r="B15" s="15"/>
-      <c r="C15" s="43" t="s">
+      <c r="C15" s="42" t="s">
         <v>98</v>
       </c>
-      <c r="D15" s="41" t="s">
+      <c r="D15" s="40" t="s">
         <v>99</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="F15" s="41" t="s">
+      <c r="F15" s="40" t="s">
         <v>101</v>
       </c>
       <c r="G15" s="11" t="s">
@@ -2606,8 +2610,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N15" s="29"/>
-      <c r="O15" s="29"/>
+      <c r="N15" s="28"/>
+      <c r="O15" s="28"/>
       <c r="P15" s="25">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2616,12 +2620,12 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="R15" s="37"/>
+      <c r="R15" s="36"/>
       <c r="S15" s="25">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="T15" s="37"/>
+      <c r="T15" s="36"/>
     </row>
     <row r="16" ht="15.75" spans="1:20">
       <c r="A16" s="7">
@@ -2631,13 +2635,13 @@
       <c r="C16" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="D16" s="41" t="s">
+      <c r="D16" s="40" t="s">
         <v>104</v>
       </c>
-      <c r="E16" s="41" t="s">
+      <c r="E16" s="40" t="s">
         <v>105</v>
       </c>
-      <c r="F16" s="41" t="s">
+      <c r="F16" s="40" t="s">
         <v>106</v>
       </c>
       <c r="G16" s="11" t="s">
@@ -2662,7 +2666,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N16" s="23" t="s">
+      <c r="N16" s="26" t="s">
         <v>30</v>
       </c>
       <c r="O16" s="25">
@@ -2683,7 +2687,7 @@
         <f t="shared" si="3"/>
         <v>1.256</v>
       </c>
-      <c r="T16" s="37"/>
+      <c r="T16" s="36"/>
     </row>
     <row r="17" ht="15.75" spans="1:20">
       <c r="A17" s="7">
@@ -2693,13 +2697,13 @@
       <c r="C17" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="D17" s="41" t="s">
+      <c r="D17" s="40" t="s">
         <v>110</v>
       </c>
-      <c r="E17" s="41" t="s">
+      <c r="E17" s="40" t="s">
         <v>111</v>
       </c>
-      <c r="F17" s="41" t="s">
+      <c r="F17" s="40" t="s">
         <v>112</v>
       </c>
       <c r="G17" s="11" t="s">
@@ -2724,7 +2728,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N17" s="23" t="s">
+      <c r="N17" s="26" t="s">
         <v>30</v>
       </c>
       <c r="O17" s="25">
@@ -2745,7 +2749,7 @@
         <f t="shared" si="3"/>
         <v>8.25</v>
       </c>
-      <c r="T17" s="38"/>
+      <c r="T17" s="37"/>
     </row>
     <row r="18" ht="15.75" spans="1:20">
       <c r="A18" s="7">
@@ -2754,16 +2758,16 @@
       <c r="B18" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="C18" s="43" t="s">
+      <c r="C18" s="42" t="s">
         <v>116</v>
       </c>
-      <c r="D18" s="41" t="s">
+      <c r="D18" s="40" t="s">
         <v>117</v>
       </c>
       <c r="E18" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="F18" s="41" t="s">
+      <c r="F18" s="40" t="s">
         <v>118</v>
       </c>
       <c r="G18" s="11" t="s">
@@ -2778,7 +2782,7 @@
       <c r="J18" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="K18" s="30">
+      <c r="K18" s="29">
         <v>1</v>
       </c>
       <c r="L18" s="22">
@@ -2788,7 +2792,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N18" s="23" t="s">
+      <c r="N18" s="26" t="s">
         <v>30</v>
       </c>
       <c r="O18" s="25">
@@ -2809,7 +2813,7 @@
         <f t="shared" si="3"/>
         <v>1.121</v>
       </c>
-      <c r="T18" s="39"/>
+      <c r="T18" s="38"/>
     </row>
     <row r="19" ht="15.75" spans="1:20">
       <c r="A19" s="7">
@@ -2819,13 +2823,13 @@
       <c r="C19" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="D19" s="40" t="s">
+      <c r="D19" s="39" t="s">
         <v>122</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="40" t="s">
+      <c r="F19" s="39" t="s">
         <v>123</v>
       </c>
       <c r="G19" s="11" t="s">
@@ -2840,7 +2844,7 @@
       <c r="J19" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="K19" s="30">
+      <c r="K19" s="29">
         <v>1</v>
       </c>
       <c r="L19" s="22">
@@ -2850,7 +2854,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N19" s="23" t="s">
+      <c r="N19" s="26" t="s">
         <v>30</v>
       </c>
       <c r="O19" s="25">
@@ -2871,23 +2875,23 @@
         <f t="shared" si="3"/>
         <v>0.155</v>
       </c>
-      <c r="T19" s="39"/>
+      <c r="T19" s="38"/>
     </row>
     <row r="20" ht="15.75" spans="1:20">
       <c r="A20" s="7">
         <v>18</v>
       </c>
       <c r="B20" s="19"/>
-      <c r="C20" s="43" t="s">
+      <c r="C20" s="42" t="s">
         <v>126</v>
       </c>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="40" t="s">
         <v>127</v>
       </c>
       <c r="E20" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="F20" s="41" t="s">
+      <c r="F20" s="40" t="s">
         <v>128</v>
       </c>
       <c r="G20" s="11" t="s">
@@ -2902,7 +2906,7 @@
       <c r="J20" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="K20" s="30">
+      <c r="K20" s="29">
         <v>1</v>
       </c>
       <c r="L20" s="22">
@@ -2912,7 +2916,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N20" s="23" t="s">
+      <c r="N20" s="26" t="s">
         <v>30</v>
       </c>
       <c r="O20" s="25">
@@ -2933,23 +2937,23 @@
         <f t="shared" si="3"/>
         <v>0.248</v>
       </c>
-      <c r="T20" s="39"/>
+      <c r="T20" s="38"/>
     </row>
     <row r="21" ht="15.75" spans="1:20">
       <c r="A21" s="7">
         <v>19</v>
       </c>
       <c r="B21" s="20"/>
-      <c r="C21" s="43" t="s">
+      <c r="C21" s="42" t="s">
         <v>130</v>
       </c>
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="40" t="s">
         <v>131</v>
       </c>
       <c r="E21" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="F21" s="41" t="s">
+      <c r="F21" s="40" t="s">
         <v>132</v>
       </c>
       <c r="G21" s="11" t="s">
@@ -2964,7 +2968,7 @@
       <c r="J21" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="K21" s="30">
+      <c r="K21" s="29">
         <v>5</v>
       </c>
       <c r="L21" s="11" t="s">
@@ -2992,7 +2996,7 @@
       <c r="S21" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="T21" s="39"/>
+      <c r="T21" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3023,7 +3027,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{cdb3d112-8688-489c-bd87-ba9c8af473f4}</x14:id>
+          <x14:id>{cd993221-8966-4a70-95a1-78e348db6a81}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3037,7 +3041,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{397039e1-9e62-4ef1-a35c-9d6ca27cf6ff}</x14:id>
+          <x14:id>{a076f2c8-98ba-47b2-bf63-4eebf46a19ba}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3051,7 +3055,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{c48074dc-3e13-47aa-9721-310de81d0939}</x14:id>
+          <x14:id>{b891dcfd-4448-437e-8894-c31c7321d958}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3080,7 +3084,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{cdb3d112-8688-489c-bd87-ba9c8af473f4}">
+          <x14:cfRule type="dataBar" id="{cd993221-8966-4a70-95a1-78e348db6a81}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -3093,7 +3097,7 @@
           <xm:sqref>P3:P20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{397039e1-9e62-4ef1-a35c-9d6ca27cf6ff}">
+          <x14:cfRule type="dataBar" id="{a076f2c8-98ba-47b2-bf63-4eebf46a19ba}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -3106,7 +3110,7 @@
           <xm:sqref>S3:S20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{c48074dc-3e13-47aa-9721-310de81d0939}">
+          <x14:cfRule type="dataBar" id="{b891dcfd-4448-437e-8894-c31c7321d958}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>